<commit_message>
Refactor RSVP form and remove Gallery section
- Updated RSVP form to include new fields: full name, place, WhatsApp number, side, relation, and guest count.
- Removed invitation code verification step and related logic.
- Enhanced validation for new fields and improved error handling.
- Removed Gallery section from the main page and deleted the GallerySection component.
- Adjusted styles for the hero card to improve mobile responsiveness.
- Updated API data handling to remove gallery-related functionality.
</commit_message>
<xml_diff>
--- a/backend/excel/wedding_database.xlsx
+++ b/backend/excel/wedding_database.xlsx
@@ -10,7 +10,6 @@
     <sheet name="Guests" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="RSVP" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Events" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gallery" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -718,43 +717,132 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>GuestID</t>
+          <t>FullName</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Place</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>WhatsappNumber</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Relation</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Coming</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Adults</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Children</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>FoodPreference</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Message</t>
-        </is>
-      </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>Guests</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>SubmittedAt</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Siva</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>+919020304370</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Bride</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Friend</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-07-03T20:25:12.745819</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Bindhu</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Madavoorpara</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>+919961059621</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Bride</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Friend</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-07-03T20:12:00.243117</t>
         </is>
       </c>
     </row>
@@ -883,171 +971,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ImageID</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>ImagePath</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>gallery-bride</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Bride Portrait</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>https://storage.googleapis.com/banani-generated-images/generated-images/89485a65-8d3e-42aa-ae78-4c945e71b559.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>gallery-groom</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Groom Portrait</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>https://storage.googleapis.com/banani-generated-images/generated-images/09879492-06cb-4e45-8d15-980194817ffe.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>gallery-couple-garden</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Garden Walk</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>https://storage.googleapis.com/banani-generated-images/generated-images/564d69bb-01c5-4877-8519-088bafef8a.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>gallery-church-interior</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Church Interior</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>https://storage.googleapis.com/banani-generated-images/generated-images/183643c1-0078-4856-891f-33dee7795aac.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>gallery-bouquet</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Bouquet</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>https://storage.googleapis.com/banani-generated-images/generated-images/f7a8d853-9a52-4d6d-a8c7-b3f0e954ea3c.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>gallery-first-kiss</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>First Kiss</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>https://storage.googleapis.com/banani-generated-images/generated-images/2daa0de7-8d51-49c9-ad67-a6a85eb8b8f8.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>gallery-flower-field</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Flower Field</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>https://storage.googleapis.com/banani-generated-images/generated-images/8a673d06-31e8-4342-9291-75307ea10417.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>gallery-family</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Family Portrait</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>https://storage.googleapis.com/banani-generated-images/generated-images/50281493-0077-44d2-8080-cf34feaee0ea.jpg</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>